<commit_message>
Removed #6 from the article list
</commit_message>
<xml_diff>
--- a/special-issue-articles-pes.xlsx
+++ b/special-issue-articles-pes.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\jcre\article-selection\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\jcre\jcre-pes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C78D9C1-F70F-4A36-972B-DA756FF5962B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B327D347-2C33-43ED-90A1-F37782EAD19C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{25F8B698-710B-47A8-B321-0466CE84E65C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="115">
   <si>
     <t>Year</t>
   </si>
@@ -177,18 +177,6 @@
   </si>
   <si>
     <t>Land Economics</t>
-  </si>
-  <si>
-    <t>https://www.aeaweb.org/articles?id=10.1257/pol.20130139</t>
-  </si>
-  <si>
-    <t>Only One Tree from Each Seed? Environmental Effectiveness and Poverty Alleviation in Mexico's Payments for Ecosystem Services Program</t>
-  </si>
-  <si>
-    <t>Jennifer M Alix-Garcia, Katharine R. E. Sims, Patricia Yanez-Pagans</t>
-  </si>
-  <si>
-    <t>American Economic Journal: Economic Policy</t>
   </si>
   <si>
     <t>https://www.openicpsr.org/openicpsr/project/114576/version/V1/view</t>
@@ -407,6 +395,21 @@
   </si>
   <si>
     <t>Privately Provided data by authors (reach out to Ryan McWay if you wish to replicate at mcway005@umn.edu)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">NOTE: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>As replicators claim articles from the list, I will be removing them to keep the selection up-to-date with the remaining articles which do not yet have a replicator. Once all articles have a replicator, I will re-open the full list for additional replication.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -438,12 +441,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -459,7 +468,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -471,15 +480,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -821,7 +826,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CBB912E-81A9-49D3-BB5D-0C14F9B5D07E}">
-  <dimension ref="A1:N19"/>
+  <dimension ref="A1:N25"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" style="3" bestFit="1" customWidth="1"/>
@@ -832,9 +837,9 @@
     <col min="6" max="6" width="13.7265625" customWidth="1"/>
     <col min="7" max="7" width="15.90625" style="3" customWidth="1"/>
     <col min="8" max="8" width="17.08984375" style="3" customWidth="1"/>
-    <col min="9" max="9" width="18.6328125" style="6" customWidth="1"/>
-    <col min="10" max="10" width="24.90625" style="6" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="24.6328125" style="7" customWidth="1"/>
+    <col min="9" max="9" width="18.6328125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="24.90625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.6328125" customWidth="1"/>
     <col min="12" max="12" width="17" style="3" customWidth="1"/>
     <col min="13" max="13" width="25.36328125" style="4" bestFit="1" customWidth="1"/>
   </cols>
@@ -864,20 +869,20 @@
       <c r="H1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="J1" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="2" t="s">
         <v>7</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>8</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
@@ -894,7 +899,7 @@
         <v>2025</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F2" t="s">
         <v>16</v>
@@ -905,20 +910,20 @@
       <c r="H2" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="I2" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K2" s="7" t="s">
+      <c r="I2" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K2" t="s">
         <v>19</v>
       </c>
       <c r="L2" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
@@ -946,20 +951,20 @@
       <c r="H3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K3" s="7" t="s">
+      <c r="I3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K3" t="s">
         <v>14</v>
       </c>
       <c r="L3" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
@@ -987,20 +992,20 @@
       <c r="H4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J4" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K4" s="7" t="s">
+      <c r="I4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K4" t="s">
         <v>26</v>
       </c>
       <c r="L4" s="3" t="s">
         <v>27</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
@@ -1008,19 +1013,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D5" s="3">
         <v>2025</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F5" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>13</v>
@@ -1028,81 +1033,81 @@
       <c r="H5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J5" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K5" s="7" t="s">
-        <v>60</v>
+      <c r="I5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K5" t="s">
+        <v>56</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" t="s">
+        <v>48</v>
+      </c>
+      <c r="C6" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="3">
+        <v>2018</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" t="s">
         <v>47</v>
-      </c>
-      <c r="C6" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="3">
-        <v>2015</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="F6" t="s">
-        <v>46</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>13</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I6" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J6" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K6" s="6" t="s">
-        <v>50</v>
+        <v>25</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K6" s="5" t="s">
+        <v>106</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B7" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="D7" s="3">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>13</v>
@@ -1110,40 +1115,40 @@
       <c r="H7" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I7" s="6" t="s">
+      <c r="I7" t="s">
+        <v>38</v>
+      </c>
+      <c r="J7" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="J7" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="K7" s="8" t="s">
-        <v>110</v>
+      <c r="K7" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="L7" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="C8" t="s">
-        <v>36</v>
+        <v>66</v>
       </c>
       <c r="D8" s="3">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>37</v>
+        <v>64</v>
       </c>
       <c r="F8" t="s">
-        <v>34</v>
+        <v>67</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>13</v>
@@ -1151,40 +1156,40 @@
       <c r="H8" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I8" s="7" t="s">
-        <v>38</v>
-      </c>
-      <c r="J8" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="K8" s="6" t="s">
+      <c r="I8" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K8" s="3" t="s">
         <v>41</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="C9" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="D9" s="3">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>68</v>
+        <v>37</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>13</v>
@@ -1192,40 +1197,40 @@
       <c r="H9" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I9" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="K9" s="6" t="s">
+      <c r="I9" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K9" s="3" t="s">
         <v>41</v>
       </c>
       <c r="L9" s="3" t="s">
         <v>33</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="B10" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>78</v>
+        <v>59</v>
       </c>
       <c r="D10" s="3">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" t="s">
-        <v>76</v>
+        <v>57</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>60</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>13</v>
@@ -1233,25 +1238,25 @@
       <c r="H10" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I10" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="K10" s="6" t="s">
+      <c r="I10" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="K10" s="3" t="s">
         <v>41</v>
       </c>
       <c r="L10" s="3" t="s">
         <v>33</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
         <v>62</v>
@@ -1260,13 +1265,13 @@
         <v>63</v>
       </c>
       <c r="D11" s="3">
-        <v>2014</v>
+        <v>2018</v>
       </c>
       <c r="E11" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" t="s">
         <v>61</v>
-      </c>
-      <c r="F11" s="1" t="s">
-        <v>64</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>13</v>
@@ -1274,163 +1279,163 @@
       <c r="H11" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I11" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="K11" s="6" t="s">
-        <v>41</v>
+      <c r="I11" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="J11" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K11" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>33</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>82</v>
       </c>
       <c r="D12" s="3">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>37</v>
+        <v>80</v>
       </c>
       <c r="F12" t="s">
-        <v>65</v>
+        <v>79</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>13</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K12" s="6" t="s">
-        <v>55</v>
+        <v>13</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>103</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>33</v>
+        <v>104</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C13" t="s">
+        <v>84</v>
+      </c>
+      <c r="D13" s="3">
+        <v>2016</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" t="s">
         <v>85</v>
-      </c>
-      <c r="C13" t="s">
-        <v>86</v>
-      </c>
-      <c r="D13" s="3">
-        <v>2019</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="F13" t="s">
-        <v>83</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>13</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J13" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K13" s="6" t="s">
-        <v>107</v>
+        <v>25</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="J13" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>51</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>108</v>
+        <v>33</v>
       </c>
       <c r="M13" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="B14" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="D14" s="3">
-        <v>2016</v>
+        <v>2012</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="F14" t="s">
-        <v>89</v>
+        <v>42</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I14" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="J14" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K14" s="6" t="s">
-        <v>55</v>
+      <c r="I14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>46</v>
       </c>
       <c r="L14" s="3" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="M14" s="4" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>30</v>
       </c>
       <c r="C15" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="D15" s="3">
-        <v>2012</v>
+        <v>2021</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="F15" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>25</v>
@@ -1438,14 +1443,14 @@
       <c r="H15" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I15" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K15" s="6" t="s">
-        <v>50</v>
+      <c r="I15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>112</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>15</v>
@@ -1456,22 +1461,22 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B16" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
       <c r="C16" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="D16" s="3">
-        <v>2021</v>
+        <v>2017</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="F16" t="s">
-        <v>29</v>
+        <v>71</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>25</v>
@@ -1479,40 +1484,40 @@
       <c r="H16" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I16" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J16" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K16" s="6" t="s">
-        <v>116</v>
+      <c r="I16" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>111</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M16" s="4" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C17" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="D17" s="3">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="F17" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>25</v>
@@ -1520,40 +1525,41 @@
       <c r="H17" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I17" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J17" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K17" s="6" t="s">
-        <v>115</v>
+      <c r="I17" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J17" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K17" s="3" t="s">
+        <v>113</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="M17" s="4" t="s">
-        <v>102</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="N17" s="3"/>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="C18" t="s">
-        <v>82</v>
+        <v>109</v>
       </c>
       <c r="D18" s="3">
         <v>2019</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
       <c r="F18" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="G18" s="3" t="s">
         <v>25</v>
@@ -1561,71 +1567,52 @@
       <c r="H18" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="I18" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J18" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K18" s="6" t="s">
-        <v>117</v>
+      <c r="I18" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="K18" s="5" t="s">
+        <v>106</v>
       </c>
       <c r="L18" s="3" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="M18" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="N18" s="3"/>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A19" s="3">
-        <v>39</v>
-      </c>
-      <c r="B19" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B23" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="C19" t="s">
-        <v>113</v>
-      </c>
-      <c r="D19" s="3">
-        <v>2019</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="F19" t="s">
-        <v>111</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="I19" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="J19" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="K19" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="L19" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="M19" s="4" t="s">
-        <v>102</v>
-      </c>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B23:E25"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="F3" r:id="rId1" xr:uid="{5FEF72A3-5737-435B-92EE-4E2A4ED27844}"/>
-    <hyperlink ref="I11" r:id="rId2" xr:uid="{2B2C98B4-32F3-48AF-8716-927CF0472219}"/>
-    <hyperlink ref="F11" r:id="rId3" xr:uid="{6D920B96-2403-4D30-88B7-0E94E06AA396}"/>
-    <hyperlink ref="K7" r:id="rId4" xr:uid="{86622696-A6B7-4A73-B69C-032D886A5019}"/>
-    <hyperlink ref="K19" r:id="rId5" xr:uid="{D93727E8-BBB3-4510-9AFA-008D20C241B1}"/>
+    <hyperlink ref="I10" r:id="rId2" xr:uid="{2B2C98B4-32F3-48AF-8716-927CF0472219}"/>
+    <hyperlink ref="F10" r:id="rId3" xr:uid="{6D920B96-2403-4D30-88B7-0E94E06AA396}"/>
+    <hyperlink ref="K6" r:id="rId4" xr:uid="{86622696-A6B7-4A73-B69C-032D886A5019}"/>
+    <hyperlink ref="K18" r:id="rId5" xr:uid="{D93727E8-BBB3-4510-9AFA-008D20C241B1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId6"/>

</xml_diff>

<commit_message>
Article #39 was claimed
</commit_message>
<xml_diff>
--- a/special-issue-articles-pes.xlsx
+++ b/special-issue-articles-pes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\jcre\jcre-pes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B327D347-2C33-43ED-90A1-F37782EAD19C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801A7794-9333-417F-9A35-89940099C609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{25F8B698-710B-47A8-B321-0466CE84E65C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="110">
   <si>
     <t>Year</t>
   </si>
@@ -138,9 +138,6 @@
   </si>
   <si>
     <t>Forest Policy and Economics</t>
-  </si>
-  <si>
-    <t>?</t>
   </si>
   <si>
     <t>https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0131544</t>
@@ -374,18 +371,6 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/1mg2-h3OuANM8Lp7m9-IUcjzvwsUoEa2U/view</t>
-  </si>
-  <si>
-    <t>https://documents1.worldbank.org/curated/en/694951547752004287/pdf/W%20PS8707.pdf</t>
-  </si>
-  <si>
-    <t>World Bank Working Paper Series</t>
-  </si>
-  <si>
-    <t>Jennifer M Alix-Garcia, Katharine Sims, Victor Hugo Orozco-Olvera, Laura Costica, Jorge David Fernandez Medina, Sofia Romo-Monroy, stefano pagiola</t>
-  </si>
-  <si>
-    <t>Can Environmental Cash Transfers Reduce Deforestation and Improve Social Outcomes? A regression discontinuity analysis of Mexico's National Program (2011 - 2014)</t>
   </si>
   <si>
     <t>Privately Provided by authors and via: https://zenodo.org/records/21281712</t>
@@ -826,7 +811,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CBB912E-81A9-49D3-BB5D-0C14F9B5D07E}">
-  <dimension ref="A1:N25"/>
+  <dimension ref="A1:N24"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" style="3" bestFit="1" customWidth="1"/>
@@ -870,10 +855,10 @@
         <v>6</v>
       </c>
       <c r="I1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="J1" s="2" t="s">
-        <v>40</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>7</v>
@@ -882,7 +867,7 @@
         <v>8</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.35">
@@ -899,7 +884,7 @@
         <v>2025</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F2" t="s">
         <v>16</v>
@@ -911,10 +896,10 @@
         <v>13</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K2" t="s">
         <v>19</v>
@@ -923,7 +908,7 @@
         <v>15</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.35">
@@ -952,10 +937,10 @@
         <v>13</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K3" t="s">
         <v>14</v>
@@ -964,7 +949,7 @@
         <v>15</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
@@ -993,10 +978,10 @@
         <v>13</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K4" t="s">
         <v>26</v>
@@ -1005,7 +990,7 @@
         <v>27</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
@@ -1013,19 +998,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C5" t="s">
         <v>54</v>
-      </c>
-      <c r="C5" t="s">
-        <v>55</v>
       </c>
       <c r="D5" s="3">
         <v>2025</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>13</v>
@@ -1034,19 +1019,19 @@
         <v>13</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="L5" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
@@ -1054,19 +1039,19 @@
         <v>7</v>
       </c>
       <c r="B6" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" t="s">
         <v>48</v>
-      </c>
-      <c r="C6" t="s">
-        <v>49</v>
       </c>
       <c r="D6" s="3">
         <v>2018</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>13</v>
@@ -1075,19 +1060,19 @@
         <v>25</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
@@ -1095,19 +1080,19 @@
         <v>9</v>
       </c>
       <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7" t="s">
         <v>35</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
       </c>
       <c r="D7" s="3">
         <v>2015</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F7" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>13</v>
@@ -1116,19 +1101,19 @@
         <v>25</v>
       </c>
       <c r="I7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
@@ -1136,19 +1121,19 @@
         <v>10</v>
       </c>
       <c r="B8" t="s">
+        <v>64</v>
+      </c>
+      <c r="C8" t="s">
         <v>65</v>
-      </c>
-      <c r="C8" t="s">
-        <v>66</v>
       </c>
       <c r="D8" s="3">
         <v>2018</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>13</v>
@@ -1157,19 +1142,19 @@
         <v>25</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
@@ -1177,19 +1162,19 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
+        <v>72</v>
+      </c>
+      <c r="C9" t="s">
         <v>73</v>
-      </c>
-      <c r="C9" t="s">
-        <v>74</v>
       </c>
       <c r="D9" s="3">
         <v>2015</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>13</v>
@@ -1198,19 +1183,19 @@
         <v>25</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
@@ -1218,19 +1203,19 @@
         <v>26</v>
       </c>
       <c r="B10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" t="s">
         <v>58</v>
-      </c>
-      <c r="C10" t="s">
-        <v>59</v>
       </c>
       <c r="D10" s="3">
         <v>2014</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>13</v>
@@ -1239,19 +1224,19 @@
         <v>25</v>
       </c>
       <c r="I10" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
@@ -1259,19 +1244,19 @@
         <v>27</v>
       </c>
       <c r="B11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C11" t="s">
         <v>62</v>
-      </c>
-      <c r="C11" t="s">
-        <v>63</v>
       </c>
       <c r="D11" s="3">
         <v>2018</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F11" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>13</v>
@@ -1280,19 +1265,19 @@
         <v>25</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
@@ -1300,19 +1285,19 @@
         <v>34</v>
       </c>
       <c r="B12" t="s">
+        <v>80</v>
+      </c>
+      <c r="C12" t="s">
         <v>81</v>
-      </c>
-      <c r="C12" t="s">
-        <v>82</v>
       </c>
       <c r="D12" s="3">
         <v>2019</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>13</v>
@@ -1321,19 +1306,19 @@
         <v>13</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K12" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="L12" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="L12" s="3" t="s">
-        <v>104</v>
-      </c>
       <c r="M12" s="4" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
@@ -1341,19 +1326,19 @@
         <v>37</v>
       </c>
       <c r="B13" t="s">
+        <v>82</v>
+      </c>
+      <c r="C13" t="s">
         <v>83</v>
-      </c>
-      <c r="C13" t="s">
-        <v>84</v>
       </c>
       <c r="D13" s="3">
         <v>2016</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G13" s="3" t="s">
         <v>13</v>
@@ -1362,19 +1347,19 @@
         <v>25</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="M13" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
@@ -1382,19 +1367,19 @@
         <v>5</v>
       </c>
       <c r="B14" t="s">
+        <v>42</v>
+      </c>
+      <c r="C14" t="s">
         <v>43</v>
-      </c>
-      <c r="C14" t="s">
-        <v>44</v>
       </c>
       <c r="D14" s="3">
         <v>2012</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>25</v>
@@ -1403,19 +1388,19 @@
         <v>25</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L14" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M14" s="4" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
@@ -1444,19 +1429,19 @@
         <v>25</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M15" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
@@ -1464,19 +1449,19 @@
         <v>31</v>
       </c>
       <c r="B16" t="s">
+        <v>68</v>
+      </c>
+      <c r="C16" t="s">
         <v>69</v>
-      </c>
-      <c r="C16" t="s">
-        <v>70</v>
       </c>
       <c r="D16" s="3">
         <v>2017</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>25</v>
@@ -1485,19 +1470,19 @@
         <v>25</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M16" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.35">
@@ -1505,19 +1490,19 @@
         <v>33</v>
       </c>
       <c r="B17" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D17" s="3">
         <v>2019</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>25</v>
@@ -1526,67 +1511,32 @@
         <v>25</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="L17" s="3" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
       <c r="M17" s="4" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="N17" s="3"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A18" s="3">
-        <v>39</v>
-      </c>
-      <c r="B18" t="s">
-        <v>110</v>
-      </c>
-      <c r="C18" t="s">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B22" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="D18" s="3">
-        <v>2019</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="F18" t="s">
-        <v>107</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="K18" s="5" t="s">
-        <v>106</v>
-      </c>
-      <c r="L18" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="M18" s="4" t="s">
-        <v>98</v>
-      </c>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B23" s="6" t="s">
-        <v>114</v>
-      </c>
+      <c r="B23" s="6"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
@@ -1597,24 +1547,17 @@
       <c r="D24" s="6"/>
       <c r="E24" s="6"/>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
-      <c r="E25" s="6"/>
-    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B23:E25"/>
+    <mergeCell ref="B22:E24"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F3" r:id="rId1" xr:uid="{5FEF72A3-5737-435B-92EE-4E2A4ED27844}"/>
     <hyperlink ref="I10" r:id="rId2" xr:uid="{2B2C98B4-32F3-48AF-8716-927CF0472219}"/>
     <hyperlink ref="F10" r:id="rId3" xr:uid="{6D920B96-2403-4D30-88B7-0E94E06AA396}"/>
     <hyperlink ref="K6" r:id="rId4" xr:uid="{86622696-A6B7-4A73-B69C-032D886A5019}"/>
-    <hyperlink ref="K18" r:id="rId5" xr:uid="{D93727E8-BBB3-4510-9AFA-008D20C241B1}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId6"/>
+  <pageSetup orientation="portrait" r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Article #27 was claimed
</commit_message>
<xml_diff>
--- a/special-issue-articles-pes.xlsx
+++ b/special-issue-articles-pes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\jcre\jcre-pes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801A7794-9333-417F-9A35-89940099C609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{301EDD8C-801A-4B6A-B681-182059824A9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{25F8B698-710B-47A8-B321-0466CE84E65C}"/>
+    <workbookView xWindow="-28920" yWindow="3780" windowWidth="29040" windowHeight="15720" xr2:uid="{25F8B698-710B-47A8-B321-0466CE84E65C}"/>
   </bookViews>
   <sheets>
     <sheet name="Articles" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="105">
   <si>
     <t>Year</t>
   </si>
@@ -221,15 +221,6 @@
     <t>http://dx.doi.org/10.1016/j.gloenvcha.2014.07.003</t>
   </si>
   <si>
-    <t>https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0200881</t>
-  </si>
-  <si>
-    <t>Do payments for forest ecosystem services generate double dividends? An integrated impact assessment of Vietnam’s PES program</t>
-  </si>
-  <si>
-    <t>Thu-Ha Dang Phan, Roy Brouwer, Long Phi Hoang, Marc David Davidson</t>
-  </si>
-  <si>
     <t>American Journal of Agricultural Economics</t>
   </si>
   <si>
@@ -297,9 +288,6 @@
   </si>
   <si>
     <t>American Economic Review: Insights</t>
-  </si>
-  <si>
-    <t>https://journals.plos.org/plosone/article?id=10.1371/journal.pone.0200881#sec019</t>
   </si>
   <si>
     <t>https://figshare.com/articles/dataset/Quindio_Silvopastoral_xlsx/2081452/1?file=3713731</t>
@@ -350,11 +338,6 @@
   <si>
     <t>Appendix A. Supplementary data
 Download all supplementary files included with this article</t>
-  </si>
-  <si>
-    <t>S1 File. Anonymized data set of the survey.
-https://doi.org/10.1371/journal.pone.0200881.s004
-(XLSX)</t>
   </si>
   <si>
     <t>Data accessibility: Data and code to reproduce analysis in this paper are
@@ -811,7 +794,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CBB912E-81A9-49D3-BB5D-0C14F9B5D07E}">
-  <dimension ref="A1:N24"/>
+  <dimension ref="A1:N23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" style="3" bestFit="1" customWidth="1"/>
@@ -829,7 +812,7 @@
     <col min="13" max="13" width="25.36328125" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>20</v>
       </c>
@@ -867,10 +850,10 @@
         <v>8</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -884,7 +867,7 @@
         <v>2025</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F2" t="s">
         <v>16</v>
@@ -908,10 +891,10 @@
         <v>15</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -949,10 +932,10 @@
         <v>15</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -990,10 +973,10 @@
         <v>27</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1031,10 +1014,10 @@
         <v>15</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>7</v>
       </c>
@@ -1066,16 +1049,16 @@
         <v>50</v>
       </c>
       <c r="K6" s="5" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="L6" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>9</v>
       </c>
@@ -1113,27 +1096,27 @@
         <v>40</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C8" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D8" s="3">
         <v>2018</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" t="s">
         <v>63</v>
-      </c>
-      <c r="F8" t="s">
-        <v>66</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>13</v>
@@ -1142,7 +1125,7 @@
         <v>25</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J8" s="3" t="s">
         <v>50</v>
@@ -1154,18 +1137,18 @@
         <v>40</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="D9" s="3">
         <v>2015</v>
@@ -1174,7 +1157,7 @@
         <v>36</v>
       </c>
       <c r="F9" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>13</v>
@@ -1183,7 +1166,7 @@
         <v>25</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="J9" s="3" t="s">
         <v>50</v>
@@ -1195,10 +1178,10 @@
         <v>40</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>26</v>
       </c>
@@ -1236,150 +1219,150 @@
         <v>40</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="B11" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="C11" t="s">
-        <v>62</v>
+        <v>78</v>
       </c>
       <c r="D11" s="3">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="F11" t="s">
-        <v>60</v>
+        <v>75</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>13</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>86</v>
+        <v>40</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>40</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>40</v>
+        <v>97</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>40</v>
+        <v>98</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" t="s">
         <v>80</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" s="3">
+        <v>2016</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" t="s">
         <v>81</v>
-      </c>
-      <c r="D12" s="3">
-        <v>2019</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="F12" t="s">
-        <v>78</v>
       </c>
       <c r="G12" s="3" t="s">
         <v>13</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>40</v>
+        <v>83</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>40</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>102</v>
+        <v>40</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>103</v>
+        <v>40</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="B13" t="s">
-        <v>82</v>
+        <v>42</v>
       </c>
       <c r="C13" t="s">
-        <v>83</v>
+        <v>43</v>
       </c>
       <c r="D13" s="3">
-        <v>2016</v>
+        <v>2012</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="F13" t="s">
-        <v>84</v>
+        <v>41</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>25</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>87</v>
+        <v>40</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>40</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="M13" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B14" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
-        <v>43</v>
+        <v>31</v>
       </c>
       <c r="D14" s="3">
-        <v>2012</v>
+        <v>2021</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>44</v>
+        <v>32</v>
       </c>
       <c r="F14" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="G14" s="3" t="s">
         <v>25</v>
@@ -1394,7 +1377,7 @@
         <v>40</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>45</v>
+        <v>102</v>
       </c>
       <c r="L14" s="3" t="s">
         <v>15</v>
@@ -1403,24 +1386,24 @@
         <v>93</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
-        <v>8</v>
+        <v>31</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>65</v>
       </c>
       <c r="C15" t="s">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="D15" s="3">
-        <v>2021</v>
+        <v>2017</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>32</v>
+        <v>44</v>
       </c>
       <c r="F15" t="s">
-        <v>29</v>
+        <v>67</v>
       </c>
       <c r="G15" s="3" t="s">
         <v>25</v>
@@ -1435,33 +1418,33 @@
         <v>40</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="L15" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M15" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C16" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D16" s="3">
-        <v>2017</v>
+        <v>2019</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>44</v>
+        <v>64</v>
       </c>
       <c r="F16" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G16" s="3" t="s">
         <v>25</v>
@@ -1476,80 +1459,39 @@
         <v>40</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="L16" s="3" t="s">
         <v>15</v>
       </c>
       <c r="M16" s="4" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A17" s="3">
-        <v>33</v>
-      </c>
-      <c r="B17" t="s">
-        <v>75</v>
-      </c>
-      <c r="C17" t="s">
-        <v>77</v>
-      </c>
-      <c r="D17" s="3">
-        <v>2019</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="F17" t="s">
-        <v>76</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="K17" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="L17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="M17" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="N17" s="3"/>
-    </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B22" s="6" t="s">
-        <v>109</v>
-      </c>
+        <v>93</v>
+      </c>
+      <c r="N16" s="3"/>
+    </row>
+    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B21" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+    </row>
+    <row r="22" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B22" s="6"/>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
       <c r="E22" s="6"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:5" x14ac:dyDescent="0.35">
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
       <c r="E23" s="6"/>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
-      <c r="E24" s="6"/>
-    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B22:E24"/>
+    <mergeCell ref="B21:E23"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="F3" r:id="rId1" xr:uid="{5FEF72A3-5737-435B-92EE-4E2A4ED27844}"/>

</xml_diff>

<commit_message>
Article #3 claimed. Removed Article #5
</commit_message>
<xml_diff>
--- a/special-issue-articles-pes.xlsx
+++ b/special-issue-articles-pes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\jcre\jcre-pes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08BCBDFD-E898-43AB-87FE-2C7A19A6C48C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBD2D279-2CC8-4B6C-98EA-A4FEF4708783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{25F8B698-710B-47A8-B321-0466CE84E65C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="79">
   <si>
     <t>Year</t>
   </si>
@@ -89,30 +89,9 @@
     <t>Rank</t>
   </si>
   <si>
-    <t>https://www.nature.com/articles/s41467-024-53643-1</t>
-  </si>
-  <si>
-    <t>Redesigning payments for ecosystem services to increase cost-effectiveness</t>
-  </si>
-  <si>
-    <t>Santiago Izquierdo-Tort, Seema Jayachandran, Santiago Saavedra</t>
-  </si>
-  <si>
-    <t>Nature Communications</t>
-  </si>
-  <si>
     <t>No</t>
   </si>
   <si>
-    <t>https://dataverse.harvard.edu/dataset.xhtml?persistentId=doi:10.7910/DVN/KYE3VT</t>
-  </si>
-  <si>
-    <t>Stata, R</t>
-  </si>
-  <si>
-    <t>No (Data Privacy)</t>
-  </si>
-  <si>
     <t>https://www.sciencedirect.com/science/article/abs/pii/S1389934121001830</t>
   </si>
   <si>
@@ -149,24 +128,9 @@
     <t>N/A</t>
   </si>
   <si>
-    <t>https://www.jstor.org/stable/23272663?seq=1</t>
-  </si>
-  <si>
-    <t>Forest Conservation and Slippage: Evidence from Mexico's National Payments for Ecosystem Services Program</t>
-  </si>
-  <si>
-    <t>Jennifer M Alix-Garcia, Elizabeth N Shapiro, Katharine R E Sims</t>
-  </si>
-  <si>
     <t>Land Economics</t>
   </si>
   <si>
-    <t>https://www.openicpsr.org/openicpsr/project/114576/version/V1/view</t>
-  </si>
-  <si>
-    <t>Need to contact authors</t>
-  </si>
-  <si>
     <t>https://direct.mit.edu/rest/article-abstract/107/5/1197/118766/Harvesting-the-Rain-The-Adoption-of-Environmental?redirectedFrom=fulltext</t>
   </si>
   <si>
@@ -269,19 +233,10 @@
     <t>Statement of Data Avaliablity</t>
   </si>
   <si>
-    <t>Data availability
-Due to the sensitive and identifiable nature of the data per the ethics approvals, the raw data is unable to be publicly shared. Please contact the corresponding authors for further details.
-Code availability
-Code is available in this link https://dataverse.harvard.edu/dataset.xhtml?persistentId=doi:10.7910/DVN/KYE3VT.</t>
-  </si>
-  <si>
     <t>Replication material by policy: https://direct.mit.edu/rest/pages/submission-guidelines</t>
   </si>
   <si>
     <t>Replication material by policy: https://www.aeaweb.org/journals/data/data-code-policy</t>
-  </si>
-  <si>
-    <t>No data or code statements</t>
   </si>
   <si>
     <t>This file contains all data necessary to replicate the underlying findings reported in this paper. https://doi.org/10.1371/journal.pone.0131544.s001</t>
@@ -758,7 +713,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CBB912E-81A9-49D3-BB5D-0C14F9B5D07E}">
-  <dimension ref="A1:N21"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" style="3" bestFit="1" customWidth="1"/>
@@ -802,10 +757,10 @@
         <v>6</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>7</v>
@@ -814,7 +769,7 @@
         <v>8</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>75</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.35">
@@ -831,7 +786,7 @@
         <v>2025</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="F2" t="s">
         <v>11</v>
@@ -843,10 +798,10 @@
         <v>9</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="K2" t="s">
         <v>14</v>
@@ -855,529 +810,447 @@
         <v>10</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>32</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>33</v>
       </c>
       <c r="D3" s="3">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="F3" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>9</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="K3" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>23</v>
       </c>
       <c r="D4" s="3">
-        <v>2025</v>
+        <v>2015</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="G4" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>35</v>
+        <v>16</v>
+      </c>
+      <c r="I4" t="s">
+        <v>25</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="K4" t="s">
-        <v>46</v>
+        <v>28</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>28</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>10</v>
+        <v>28</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>77</v>
+        <v>66</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>41</v>
       </c>
       <c r="D5" s="3">
-        <v>2015</v>
+        <v>2018</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="G5" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I5" t="s">
-        <v>32</v>
+        <v>16</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>42</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D6" s="3">
-        <v>2018</v>
+        <v>2015</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="F6" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="G6" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="M6" s="4" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="B7" t="s">
-        <v>60</v>
+        <v>36</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>37</v>
       </c>
       <c r="D7" s="3">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="F7" t="s">
-        <v>59</v>
+        <v>35</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>38</v>
       </c>
       <c r="G7" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>62</v>
+        <v>16</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>38</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="M7" s="4" t="s">
-        <v>83</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="D8" s="3">
-        <v>2014</v>
+        <v>2019</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>50</v>
+        <v>55</v>
+      </c>
+      <c r="F8" t="s">
+        <v>54</v>
       </c>
       <c r="G8" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>50</v>
+        <v>9</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>28</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>41</v>
+        <v>28</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>35</v>
+        <v>72</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>35</v>
+        <v>73</v>
       </c>
       <c r="M8" s="4" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B9" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="C9" t="s">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="D9" s="3">
-        <v>2019</v>
+        <v>2016</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>67</v>
+        <v>24</v>
       </c>
       <c r="F9" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="G9" s="3" t="s">
         <v>9</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>35</v>
+        <v>62</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>86</v>
+        <v>28</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>87</v>
+        <v>28</v>
       </c>
       <c r="M9" s="4" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
-        <v>37</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>70</v>
+        <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>71</v>
+        <v>19</v>
       </c>
       <c r="D10" s="3">
-        <v>2016</v>
+        <v>2021</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="F10" t="s">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>74</v>
+        <v>28</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>35</v>
+        <v>76</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>35</v>
+        <v>10</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>88</v>
+        <v>68</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>44</v>
       </c>
       <c r="C11" t="s">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="D11" s="3">
-        <v>2012</v>
+        <v>2017</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="F11" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>40</v>
+        <v>75</v>
       </c>
       <c r="L11" s="3" t="s">
         <v>10</v>
       </c>
       <c r="M11" s="4" t="s">
-        <v>79</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="B12" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="C12" t="s">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="D12" s="3">
-        <v>2021</v>
+        <v>2019</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="F12" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>90</v>
+        <v>77</v>
       </c>
       <c r="L12" s="3" t="s">
         <v>10</v>
       </c>
       <c r="M12" s="4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A13" s="3">
-        <v>31</v>
-      </c>
-      <c r="B13" t="s">
-        <v>56</v>
-      </c>
-      <c r="C13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D13" s="3">
-        <v>2017</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="L13" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="M13" s="4" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
-      <c r="A14" s="3">
-        <v>33</v>
-      </c>
-      <c r="B14" t="s">
-        <v>63</v>
-      </c>
-      <c r="C14" t="s">
-        <v>65</v>
-      </c>
-      <c r="D14" s="3">
-        <v>2019</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F14" t="s">
-        <v>64</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="M14" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="N14" s="3"/>
+        <v>68</v>
+      </c>
+      <c r="N12" s="3"/>
+    </row>
+    <row r="17" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B17" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+    </row>
+    <row r="18" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B19" s="6" t="s">
-        <v>92</v>
-      </c>
+      <c r="B19" s="6"/>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
       <c r="E19" s="6"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B20" s="6"/>
-      <c r="C20" s="6"/>
-      <c r="D20" s="6"/>
-      <c r="E20" s="6"/>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.35">
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
-      <c r="E21" s="6"/>
-    </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B19:E21"/>
+    <mergeCell ref="B17:E19"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="I8" r:id="rId1" xr:uid="{2B2C98B4-32F3-48AF-8716-927CF0472219}"/>
-    <hyperlink ref="F8" r:id="rId2" xr:uid="{6D920B96-2403-4D30-88B7-0E94E06AA396}"/>
+    <hyperlink ref="I7" r:id="rId1" xr:uid="{2B2C98B4-32F3-48AF-8716-927CF0472219}"/>
+    <hyperlink ref="F7" r:id="rId2" xr:uid="{6D920B96-2403-4D30-88B7-0E94E06AA396}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId3"/>

</xml_diff>

<commit_message>
Article #21 added - replication packet received
</commit_message>
<xml_diff>
--- a/special-issue-articles-pes.xlsx
+++ b/special-issue-articles-pes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\jcre\jcre-pes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40524860-2430-481D-8A95-B541DAAA95B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2009B77-7220-4726-95FA-ED1A038FE359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="3780" windowWidth="29040" windowHeight="15720" xr2:uid="{25F8B698-710B-47A8-B321-0466CE84E65C}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="64">
   <si>
     <t>Year</t>
   </si>
@@ -239,6 +239,18 @@
       </rPr>
       <t>As replicators claim articles from the list, I will be removing them to keep the selection up-to-date with the remaining articles which do not yet have a replicator. Once all articles have a replicator, I will re-open the full list for additional replication.</t>
     </r>
+  </si>
+  <si>
+    <t>Do Payments for Environmental Services Affect Forest Cover? A Farm-Level Evaluation from Costa Rica</t>
+  </si>
+  <si>
+    <t>Rodrigo A Arriagada, Paul J Ferraro, Erin O Sills, Subhrendu K Pattanayak, Silvia Cordero-Sancho</t>
+  </si>
+  <si>
+    <t>https://le.uwpress.org/content/88/2/382.short</t>
+  </si>
+  <si>
+    <t>Stata, R</t>
   </si>
 </sst>
 </file>
@@ -655,7 +667,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CBB912E-81A9-49D3-BB5D-0C14F9B5D07E}">
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:T16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="10.453125" style="3" bestFit="1" customWidth="1"/>
@@ -673,7 +685,7 @@
     <col min="13" max="13" width="25.36328125" style="4" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="2" t="s">
         <v>11</v>
       </c>
@@ -714,7 +726,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>9</v>
       </c>
@@ -755,7 +767,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>10</v>
       </c>
@@ -796,7 +808,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>15</v>
       </c>
@@ -837,7 +849,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>26</v>
       </c>
@@ -878,7 +890,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>37</v>
       </c>
@@ -919,7 +931,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>8</v>
       </c>
@@ -960,7 +972,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>31</v>
       </c>
@@ -1001,7 +1013,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>33</v>
       </c>
@@ -1043,7 +1055,52 @@
       </c>
       <c r="N9" s="3"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A10" s="3">
+        <v>21</v>
+      </c>
+      <c r="B10" t="s">
+        <v>60</v>
+      </c>
+      <c r="C10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D10" s="3">
+        <v>2012</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="L10" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="M10" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="R10" s="3"/>
+      <c r="T10" s="4"/>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B14" s="6" t="s">
         <v>59</v>
       </c>
@@ -1051,13 +1108,13 @@
       <c r="D14" s="6"/>
       <c r="E14" s="6"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
       <c r="D15" s="6"/>
       <c r="E15" s="6"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
       <c r="D16" s="6"/>

</xml_diff>

<commit_message>
Articles 21 and 26 claimed
</commit_message>
<xml_diff>
--- a/special-issue-articles-pes.xlsx
+++ b/special-issue-articles-pes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\jcre\jcre-pes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2009B77-7220-4726-95FA-ED1A038FE359}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EF58289-E7AB-42B3-B988-F2904792E7C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="3780" windowWidth="29040" windowHeight="15720" xr2:uid="{25F8B698-710B-47A8-B321-0466CE84E65C}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{25F8B698-710B-47A8-B321-0466CE84E65C}"/>
   </bookViews>
   <sheets>
     <sheet name="Articles" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="55">
   <si>
     <t>Year</t>
   </si>
@@ -117,18 +117,6 @@
   </si>
   <si>
     <t>Land Economics</t>
-  </si>
-  <si>
-    <t>Global Environmental Change</t>
-  </si>
-  <si>
-    <t>Measuring effectiveness, efficiency and equity in an experimental Payments for Ecosystem Services trial</t>
-  </si>
-  <si>
-    <t>Adrian Martin, Nicole Gross-Camp, Bereket Kebede, Shawn McGuire</t>
-  </si>
-  <si>
-    <t>http://dx.doi.org/10.1016/j.gloenvcha.2014.07.003</t>
   </si>
   <si>
     <t>American Journal of Agricultural Economics</t>
@@ -208,10 +196,6 @@
 (DOC)
 S2 File. Data generated by the authors.
 https://doi.org/10.1371/journal.pone.0119881.s002</t>
-  </si>
-  <si>
-    <t>Appendix A. Supplementary data
-Download all supplementary files included with this article</t>
   </si>
   <si>
     <t>Data Availability: All relevant data are available via Figshare (https://dx.doi.org/10.6084/m9.figshare.2081452.v1)</t>
@@ -240,24 +224,12 @@
       <t>As replicators claim articles from the list, I will be removing them to keep the selection up-to-date with the remaining articles which do not yet have a replicator. Once all articles have a replicator, I will re-open the full list for additional replication.</t>
     </r>
   </si>
-  <si>
-    <t>Do Payments for Environmental Services Affect Forest Cover? A Farm-Level Evaluation from Costa Rica</t>
-  </si>
-  <si>
-    <t>Rodrigo A Arriagada, Paul J Ferraro, Erin O Sills, Subhrendu K Pattanayak, Silvia Cordero-Sancho</t>
-  </si>
-  <si>
-    <t>https://le.uwpress.org/content/88/2/382.short</t>
-  </si>
-  <si>
-    <t>Stata, R</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -269,14 +241,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -305,13 +269,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -321,15 +283,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -667,67 +625,67 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CBB912E-81A9-49D3-BB5D-0C14F9B5D07E}">
-  <dimension ref="A1:T16"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.453125" style="2" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.90625" customWidth="1"/>
     <col min="3" max="3" width="20.90625" customWidth="1"/>
-    <col min="4" max="4" width="9" style="3" customWidth="1"/>
-    <col min="5" max="5" width="45.1796875" style="3" customWidth="1"/>
+    <col min="4" max="4" width="9" style="2" customWidth="1"/>
+    <col min="5" max="5" width="45.1796875" style="2" customWidth="1"/>
     <col min="6" max="6" width="13.7265625" customWidth="1"/>
-    <col min="7" max="7" width="15.90625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="17.08984375" style="3" customWidth="1"/>
-    <col min="9" max="9" width="18.6328125" style="3" customWidth="1"/>
-    <col min="10" max="10" width="24.90625" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.90625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="17.08984375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="18.6328125" style="2" customWidth="1"/>
+    <col min="10" max="10" width="24.90625" style="2" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="24.6328125" customWidth="1"/>
-    <col min="12" max="12" width="17" style="3" customWidth="1"/>
-    <col min="13" max="13" width="25.36328125" style="4" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17" style="2" customWidth="1"/>
+    <col min="13" max="13" width="25.36328125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" s="2" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="2" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="I1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="J1" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="M1" s="2" t="s">
-        <v>49</v>
+      <c r="M1" s="1" t="s">
+        <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A2" s="3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
         <v>9</v>
       </c>
       <c r="B2" t="s">
@@ -736,399 +694,309 @@
       <c r="C2" t="s">
         <v>19</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="2">
         <v>2015</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="F2" t="s">
         <v>17</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="2" t="s">
         <v>12</v>
       </c>
       <c r="I2" t="s">
         <v>21</v>
       </c>
-      <c r="J2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="M2" s="4" t="s">
+      <c r="J2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="2">
+        <v>2018</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="2">
+        <v>2015</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D5" s="2">
+        <v>2016</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M5" s="3" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A3" s="3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <v>8</v>
+      </c>
+      <c r="B6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="2">
+        <v>2021</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B3" t="s">
+      <c r="M6" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A7" s="2">
         <v>31</v>
       </c>
-      <c r="C3" t="s">
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="3">
-        <v>2018</v>
-      </c>
-      <c r="E3" s="3" t="s">
+      <c r="D7" s="2">
+        <v>2017</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F7" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <v>33</v>
+      </c>
+      <c r="B8" t="s">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="2">
+        <v>2019</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="F3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H3" s="3" t="s">
+      <c r="F8" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="I3" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L3" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="M3" s="4" t="s">
-        <v>51</v>
-      </c>
+      <c r="H8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="N8" s="2"/>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A4" s="3">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>39</v>
-      </c>
-      <c r="C4" t="s">
-        <v>40</v>
-      </c>
-      <c r="D4" s="3">
-        <v>2015</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F4" t="s">
-        <v>38</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I4" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L4" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="M4" s="4" t="s">
-        <v>53</v>
-      </c>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B12" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A5" s="3">
-        <v>26</v>
-      </c>
-      <c r="B5" t="s">
-        <v>27</v>
-      </c>
-      <c r="C5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" s="3">
-        <v>2014</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="M5" s="4" t="s">
-        <v>54</v>
-      </c>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A6" s="3">
-        <v>37</v>
-      </c>
-      <c r="B6" t="s">
-        <v>45</v>
-      </c>
-      <c r="C6" t="s">
-        <v>46</v>
-      </c>
-      <c r="D6" s="3">
-        <v>2016</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="L6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A7" s="3">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="3">
-        <v>2021</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="L7" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A8" s="3">
-        <v>31</v>
-      </c>
-      <c r="B8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="3">
-        <v>2017</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F8" t="s">
-        <v>37</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="M8" s="4" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A9" s="3">
-        <v>33</v>
-      </c>
-      <c r="B9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="3">
-        <v>2019</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="F9" t="s">
-        <v>43</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="M9" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="N9" s="3"/>
-    </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A10" s="3">
-        <v>21</v>
-      </c>
-      <c r="B10" t="s">
-        <v>60</v>
-      </c>
-      <c r="C10" t="s">
-        <v>61</v>
-      </c>
-      <c r="D10" s="3">
-        <v>2012</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="F10" t="s">
-        <v>62</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="M10" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="R10" s="3"/>
-      <c r="T10" s="4"/>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="B14" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-    </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="B16" s="6"/>
-      <c r="C16" s="6"/>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.35">
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B14:E16"/>
+    <mergeCell ref="B12:E14"/>
   </mergeCells>
-  <hyperlinks>
-    <hyperlink ref="I5" r:id="rId1" xr:uid="{2B2C98B4-32F3-48AF-8716-927CF0472219}"/>
-    <hyperlink ref="F5" r:id="rId2" xr:uid="{6D920B96-2403-4D30-88B7-0E94E06AA396}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" r:id="rId3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>